<commit_message>
Update project document status labels
</commit_message>
<xml_diff>
--- a/public/uploads/project-docs/base-chain-planning.xlsx
+++ b/public/uploads/project-docs/base-chain-planning.xlsx
@@ -4899,7 +4899,7 @@
     <row r="2" ht="21.75" customHeight="1" s="404">
       <c r="A2" s="406" t="inlineStr">
         <is>
-          <t>2026.03 ~ 진행 중 기준  |  MVP 범위 = 야구 경기 예매부터 NFT 티켓, QR 검표, 공식 재판매까지 이어지는 상태 흐름</t>
+          <t>2026.03 ~ 고도화 중 기준  |  MVP 범위 = 야구 경기 예매부터 NFT 티켓, QR 검표, 공식 재판매까지 이어지는 상태 흐름</t>
         </is>
       </c>
     </row>
@@ -4998,7 +4998,7 @@
       </c>
       <c r="I4" s="421" t="inlineStr">
         <is>
-          <t>진행 중</t>
+          <t>고도화 중</t>
         </is>
       </c>
       <c r="J4" s="422" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="I5" s="421" t="inlineStr">
         <is>
-          <t>진행 중</t>
+          <t>고도화 중</t>
         </is>
       </c>
       <c r="J5" s="428" t="inlineStr"/>
@@ -5098,7 +5098,7 @@
       </c>
       <c r="I6" s="421" t="inlineStr">
         <is>
-          <t>진행 중</t>
+          <t>고도화 중</t>
         </is>
       </c>
       <c r="J6" s="422" t="inlineStr"/>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="I7" s="421" t="inlineStr">
         <is>
-          <t>진행 중</t>
+          <t>고도화 중</t>
         </is>
       </c>
       <c r="J7" s="428" t="inlineStr"/>
@@ -5194,7 +5194,7 @@
       </c>
       <c r="I8" s="421" t="inlineStr">
         <is>
-          <t>진행 중</t>
+          <t>고도화 중</t>
         </is>
       </c>
       <c r="J8" s="422" t="inlineStr"/>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="I9" s="421" t="inlineStr">
         <is>
-          <t>진행 중</t>
+          <t>고도화 중</t>
         </is>
       </c>
       <c r="J9" s="428" t="inlineStr"/>
@@ -5290,7 +5290,7 @@
       </c>
       <c r="I10" s="421" t="inlineStr">
         <is>
-          <t>진행 중</t>
+          <t>고도화 중</t>
         </is>
       </c>
       <c r="J10" s="422" t="inlineStr"/>
@@ -5338,7 +5338,7 @@
       </c>
       <c r="I11" s="421" t="inlineStr">
         <is>
-          <t>진행 중</t>
+          <t>고도화 중</t>
         </is>
       </c>
       <c r="J11" s="428" t="inlineStr"/>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="I12" s="421" t="inlineStr">
         <is>
-          <t>진행 중</t>
+          <t>고도화 중</t>
         </is>
       </c>
       <c r="J12" s="422" t="inlineStr"/>
@@ -5434,7 +5434,7 @@
       </c>
       <c r="I13" s="421" t="inlineStr">
         <is>
-          <t>진행 중</t>
+          <t>고도화 중</t>
         </is>
       </c>
       <c r="J13" s="428" t="inlineStr"/>
@@ -6254,7 +6254,7 @@
     <row r="1" ht="33.75" customHeight="1" s="404">
       <c r="A1" s="457" t="inlineStr">
         <is>
-          <t>BASE CHAIN - 블록체인 야구 티켓팅 플랫폼  |  개발 일정표 (2026.03 ~ 진행 중)</t>
+          <t>BASE CHAIN - 블록체인 야구 티켓팅 플랫폼  |  개발 일정표 (2026.03 ~ 고도화 중)</t>
         </is>
       </c>
     </row>
@@ -6867,7 +6867,7 @@
     <row r="2" ht="19.5" customHeight="1" s="404">
       <c r="A2" s="503" t="inlineStr">
         <is>
-          <t>프로젝트 성격에 맞춘 역할과 산출물 정리  |  기간: 2026.03 ~ 진행 중</t>
+          <t>프로젝트 성격에 맞춘 역할과 산출물 정리  |  기간: 2026.03 ~ 고도화 중</t>
         </is>
       </c>
     </row>
@@ -9475,7 +9475,7 @@
       </c>
       <c r="L5" s="768" t="inlineStr">
         <is>
-          <t>진행중</t>
+          <t>고도화 중</t>
         </is>
       </c>
     </row>
@@ -9523,7 +9523,7 @@
       </c>
       <c r="L6" s="768" t="inlineStr">
         <is>
-          <t>진행중</t>
+          <t>고도화 중</t>
         </is>
       </c>
     </row>
@@ -9571,7 +9571,7 @@
       </c>
       <c r="L7" s="788" t="inlineStr">
         <is>
-          <t>진행중</t>
+          <t>고도화 중</t>
         </is>
       </c>
     </row>
@@ -9901,7 +9901,7 @@
       <c r="K4" s="681" t="n"/>
       <c r="L4" s="768" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>점검</t>
         </is>
       </c>
       <c r="M4" s="817" t="inlineStr">
@@ -9911,7 +9911,7 @@
       </c>
       <c r="N4" s="768" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>고도화 중</t>
         </is>
       </c>
     </row>
@@ -9951,7 +9951,7 @@
       <c r="K5" s="681" t="n"/>
       <c r="L5" s="768" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>점검</t>
         </is>
       </c>
       <c r="M5" s="820" t="inlineStr">
@@ -9961,7 +9961,7 @@
       </c>
       <c r="N5" s="768" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>고도화 중</t>
         </is>
       </c>
     </row>
@@ -10001,7 +10001,7 @@
       <c r="K6" s="681" t="n"/>
       <c r="L6" s="768" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>점검</t>
         </is>
       </c>
       <c r="M6" s="822" t="inlineStr">
@@ -10011,7 +10011,7 @@
       </c>
       <c r="N6" s="768" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>고도화 중</t>
         </is>
       </c>
     </row>
@@ -10051,7 +10051,7 @@
       <c r="K7" s="681" t="n"/>
       <c r="L7" s="768" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>점검</t>
         </is>
       </c>
       <c r="M7" s="820" t="inlineStr">
@@ -10061,7 +10061,7 @@
       </c>
       <c r="N7" s="768" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>고도화 중</t>
         </is>
       </c>
     </row>
@@ -10111,7 +10111,7 @@
       </c>
       <c r="N8" s="788" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>고도화 중</t>
         </is>
       </c>
     </row>
@@ -10161,7 +10161,7 @@
       </c>
       <c r="N9" s="788" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>고도화 중</t>
         </is>
       </c>
     </row>

</xml_diff>